<commit_message>
Add footer, header blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (13):
- blocks/footer/footer.css
- blocks/footer/footer.js
- blocks/header/header.css
- blocks/header/header.js
- scripts/scripts.js
- styles/brand.css
- styles/styles.css
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/page-templates.json
- tools/importer/parsers/hero-campaign.js
- tools/importer/reports/es/es/h/home.report.json
- tools/importer/reports/import-homepage.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>es/es/h/home.report.json</t>
   </si>
   <si>
-    <t>["hero-campaign","hero-branded","columns-category","columns-category"]</t>
+    <t>["hero-campaign","hero-campaign","hero-campaign","hero-campaign","hero-campaign","hero-campaign","hero-branded","columns-category","columns-category"]</t>
   </si>
   <si>
     <t>es/es/h/home</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-06-04T13:54:40.389Z</t>
+    <t>2026-06-04T15:41:12.228Z</t>
   </si>
   <si>
     <t>Moda de Home 2026 | Mango Home España (Península y Baleares)</t>

</xml_diff>